<commit_message>
Development 2, complete the backend. Start to build the frontend.
</commit_message>
<xml_diff>
--- a/data/exports/documents.xlsx
+++ b/data/exports/documents.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,11 @@
           <t>chunks_jsonl</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>content_signature</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -486,7 +491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Digital Trends Africa 2025</t>
+          <t>Measuring digital development</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,10 +516,10 @@
         <v>56</v>
       </c>
       <c r="H2" t="n">
-        <v>100299</v>
+        <v>97782</v>
       </c>
       <c r="I2" t="n">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -529,6 +534,11 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>E:\MyProjects\ITUassistant\data\chunks\digital_trends_africa_2025.jsonl</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>661bce6487083557a7e12b8afd5e36e5</t>
         </is>
       </c>
     </row>
@@ -540,7 +550,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Facts 2022</t>
+          <t>al development: Facts and figures 202</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -565,10 +575,10 @@
         <v>36</v>
       </c>
       <c r="H3" t="n">
-        <v>48086</v>
+        <v>46494</v>
       </c>
       <c r="I3" t="n">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -583,6 +593,11 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>E:\MyProjects\ITUassistant\data\chunks\facts_2022.jsonl</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>535b9b93de7fe1bc97770ed91600affc</t>
         </is>
       </c>
     </row>
@@ -594,7 +609,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Facts 2023</t>
+          <t>Measuring digital development</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -619,10 +634,10 @@
         <v>38</v>
       </c>
       <c r="H4" t="n">
-        <v>60280</v>
+        <v>58499</v>
       </c>
       <c r="I4" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -637,18 +652,23 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>E:\MyProjects\ITUassistant\data\chunks\facts_2023.jsonl</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>836461fb4e881a0e6ff683b835736056</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>facts_2023_un.pdf</t>
+          <t>facts_2024.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Facts 2023 Un</t>
+          <t>Measuring digital development</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -662,7 +682,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -670,39 +690,44 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H5" t="n">
-        <v>60280</v>
+        <v>59931</v>
       </c>
       <c r="I5" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\facts_2023_un.pdf</t>
+          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\facts_2024.pdf</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\parsed\facts_2023_un.json</t>
+          <t>E:\MyProjects\ITUassistant\data\parsed\facts_2024.json</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\chunks\facts_2023_un.jsonl</t>
+          <t>E:\MyProjects\ITUassistant\data\chunks\facts_2024.jsonl</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>82400bf02f3e0aa4db6b0caad661726e</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>facts_2024.pdf</t>
+          <t>itu_annual_report_2024.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Facts 2024</t>
+          <t>Annual Report on the</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -712,7 +737,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>statistics_report</t>
+          <t>annual_report</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -724,39 +749,44 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="H6" t="n">
-        <v>63233</v>
+        <v>148204</v>
       </c>
       <c r="I6" t="n">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\facts_2024.pdf</t>
+          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\itu_annual_report_2024.pdf</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\parsed\facts_2024.json</t>
+          <t>E:\MyProjects\ITUassistant\data\parsed\itu_annual_report_2024.json</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\chunks\facts_2024.jsonl</t>
+          <t>E:\MyProjects\ITUassistant\data\chunks\itu_annual_report_2024.jsonl</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>7dd250d2e5a597b7a49e613f0f82d3d9</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>facts_2024_un.pdf</t>
+          <t>mdd_2024_lldc.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Facts 2024 Un</t>
+          <t>Measuring digital development</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -766,7 +796,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>statistics_report</t>
+          <t>report</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -778,135 +808,32 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H7" t="n">
-        <v>63233</v>
+        <v>67569</v>
       </c>
       <c r="I7" t="n">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\facts_2024_un.pdf</t>
+          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\mdd_2024_lldc.pdf</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\parsed\facts_2024_un.json</t>
+          <t>E:\MyProjects\ITUassistant\data\parsed\mdd_2024_lldc.json</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>E:\MyProjects\ITUassistant\data\chunks\facts_2024_un.jsonl</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>itu_annual_report_2024.pdf</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Itu Annual Report 2024</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>ITU</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>annual_report</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>72</v>
-      </c>
-      <c r="H8" t="n">
-        <v>151854</v>
-      </c>
-      <c r="I8" t="n">
-        <v>65</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\itu_annual_report_2024.pdf</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>E:\MyProjects\ITUassistant\data\parsed\itu_annual_report_2024.json</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>E:\MyProjects\ITUassistant\data\chunks\itu_annual_report_2024.jsonl</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>mdd_2024_lldc.pdf</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Mdd 2024 Lldc</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ITU</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>39</v>
-      </c>
-      <c r="H9" t="n">
-        <v>69632</v>
-      </c>
-      <c r="I9" t="n">
-        <v>38</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>E:\MyProjects\ITUassistant\data\itu_pdfs\mdd_2024_lldc.pdf</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>E:\MyProjects\ITUassistant\data\parsed\mdd_2024_lldc.json</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
           <t>E:\MyProjects\ITUassistant\data\chunks\mdd_2024_lldc.jsonl</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>3974628a4961873983ad7cb2347c381d</t>
         </is>
       </c>
     </row>

</xml_diff>